<commit_message>
Corrige rótulos dos grupos da Etapa 1
</commit_message>
<xml_diff>
--- a/kobo/gestores_diagnostico_completo.xlsx
+++ b/kobo/gestores_diagnostico_completo.xlsx
@@ -2180,7 +2180,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Água, esgoto e resíduos — local</t>
+          <t>Água, esgoto e resíduos — escola</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Responda com base na sua visão geral das locais da rede/região de atuação. Estimativas são bem-vindas; "Não sabe" é uma resposta válida e vira lacuna de conhecimento registrada.</t>
+          <t>Responda com base na sua visão geral das escolas da rede/região de atuação. Estimativas são bem-vindas; "Não sabe" é uma resposta válida e vira lacuna de conhecimento registrada.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>

</xml_diff>